<commit_message>
feature/fsel-4793: Update Export Learning Progress Report
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/BaoCaoReportStudentEvent.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/BaoCaoReportStudentEvent.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PhanPhuc\Fsel\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759C9139-E3BE-418C-B29C-9D780EDD10DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4969750-EB2B-4866-9C80-0E1C669F4D7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AA20440B-2029-433B-B2D2-6252C6B3534C}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AA20440B-2029-433B-B2D2-6252C6B3534C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>STT</t>
   </si>
@@ -91,6 +91,12 @@
   </si>
   <si>
     <t>Lesson 5</t>
+  </si>
+  <si>
+    <t>UserName</t>
+  </si>
+  <si>
+    <t>Trạng Thái</t>
   </si>
 </sst>
 </file>
@@ -206,12 +212,21 @@
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -220,15 +235,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -547,132 +553,144 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0082E27F-1FDE-4DA7-9407-00CD9A380099}">
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.25" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.25" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.25" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.375" customWidth="1"/>
+    <col min="15" max="15" width="11.375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="L1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="M1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="N1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="O1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="P1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="4"/>
-      <c r="P1" s="5" t="s">
+      <c r="Q1" s="7"/>
+      <c r="R1" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="U1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="W1" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="7"/>
-      <c r="N2" s="8" t="s">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="Q2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="P2" s="9"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="6"/>
+      <c r="R2" s="9"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="3"/>
+      <c r="V2" s="3"/>
+      <c r="W2" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="T1:T2"/>
-    <mergeCell ref="U1:U2"/>
-    <mergeCell ref="M1:M2"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="P1:P2"/>
-    <mergeCell ref="Q1:Q2"/>
-    <mergeCell ref="R1:R2"/>
-    <mergeCell ref="S1:S2"/>
+  <mergeCells count="22">
+    <mergeCell ref="N1:N2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
     <mergeCell ref="G1:G2"/>
+    <mergeCell ref="C1:C2"/>
     <mergeCell ref="H1:H2"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="J1:J2"/>
+    <mergeCell ref="L1:L2"/>
+    <mergeCell ref="M1:M2"/>
     <mergeCell ref="K1:K2"/>
-    <mergeCell ref="L1:L2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="V1:V2"/>
+    <mergeCell ref="W1:W2"/>
+    <mergeCell ref="O1:O2"/>
+    <mergeCell ref="P1:Q1"/>
+    <mergeCell ref="R1:R2"/>
+    <mergeCell ref="S1:S2"/>
+    <mergeCell ref="T1:T2"/>
+    <mergeCell ref="U1:U2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>